<commit_message>
Update Tier D FMV estimates with research-backed values
Notable changes: Yao Pristine Refractor BGS 9.5 $40->$600 (CSG 9.5
listed ~$970), VJ Edgecombe Blue Ice SGC 10 $120->$400, Paolo
Banchero Recon $50->$175, Yao Crusade $60->$200.

https://claude.ai/code/session_01GTThiDtMm869wgd52PwWVn
</commit_message>
<xml_diff>
--- a/Inventory/Goldin_Auction_FMV.xlsx
+++ b/Inventory/Goldin_Auction_FMV.xlsx
@@ -2745,10 +2745,10 @@
         <v>34</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>0.765</v>
+        <v>4.882352941176471</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Crusade Green &amp; Gold /25 PSA 10; Yao HOF</t>
+          <t>Yao low-numbered Panini inserts (Optic Gold /10 PSA 10) list $150-300; Crusade desirable insert</t>
         </is>
       </c>
     </row>
@@ -2784,10 +2784,10 @@
         <v>16</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>40</v>
+        <v>600</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>1.5</v>
+        <v>36.5</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2796,12 +2796,12 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Topps Pristine Refractor BGS 9.5; vintage Yao</t>
+          <t>CSG 9.5 copies listed ~$970 retail; BGS 9.5 slight premium; sold likely $500-700</t>
         </is>
       </c>
     </row>
@@ -2835,12 +2835,12 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Med-High</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Panini VIP card PSA 8; CC demand strong</t>
+          <t>PSA auction: 2024 VIP Gold CC PSA 8 sold $75 on eBay (Jan 2025)</t>
         </is>
       </c>
     </row>
@@ -2862,10 +2862,10 @@
         <v>26</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>0.9229999999999999</v>
+        <v>5.730769230769231</v>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
@@ -2874,12 +2874,12 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Recon Purple /25 PSA 8 w/10 auto; Paolo upside</t>
+          <t>Banchero autos /25-75 mid-tier products $100-250; PSA 8 card grade notable discount</t>
         </is>
       </c>
     </row>
@@ -2901,24 +2901,24 @@
         <v>52</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="F61" s="7" t="n">
-        <v>0.442</v>
+        <v>125</v>
+      </c>
+      <c r="F61" s="5" t="n">
+        <v>1.403846153846154</v>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Panini Instant /99; draft prospect hype</t>
+          <t>Panini Instant auto /99 draft night cards sold $100-150 raw on eBay; #3 pick</t>
         </is>
       </c>
     </row>
@@ -2940,10 +2940,10 @@
         <v>75</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0.6</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
@@ -2952,12 +2952,12 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low-Med</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Prizm Draft Picks Blue Ice /75 SGC 10; prospect premium</t>
+          <t>Penmanship Purple Ice /99 PSA 10 comps strong; Blue Ice /75 scarcer; SGC 10/10 premium</t>
         </is>
       </c>
     </row>
@@ -2979,10 +2979,10 @@
         <v>22</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>1.045</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Bowman U Purple /25 PSA 9; women's basketball rising</t>
+          <t>Raw Bowman U Purple /25 sold ~$11.50; PSA 9 ~3-4x raw; women's cards soft outside CC</t>
         </is>
       </c>
     </row>
@@ -3070,10 +3070,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Tier B FMV estimates with detailed research comps
Key changes: Ant Edwards Optic Choice $1.1K->$2K, Ant Flawless Ruby
$1.2K->$2.5K, Kobe/MJ Dual $1.5K->$2.5K, Curry Regalia $800->$1.5K,
Curry One&One $350->$1.5K. Some cards now show as PASS: Yao Mother
Lode ($575 bid vs $300 FMV), Giannis All Kings ($475 vs $300).

https://claude.ai/code/session_01GTThiDtMm869wgd52PwWVn
</commit_message>
<xml_diff>
--- a/Inventory/Goldin_Auction_FMV.xlsx
+++ b/Inventory/Goldin_Auction_FMV.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +55,9 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font/>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +106,12 @@
         <bgColor rgb="00F3E5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -156,6 +163,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -873,14 +884,14 @@
         <v>910</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>0.319</v>
+        <v>1500</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.6483516483516484</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -890,7 +901,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Top 2025 draft pick; Bowman Chrome autos hot; recent PSA 10 comps ~$1,000-1,500</t>
+          <t>Base prospect auto raw sold $1,000 (Dec 2025); PSA 10 premium; Superfractor 1/1 PSA 10 sold $18K</t>
         </is>
       </c>
     </row>
@@ -912,14 +923,14 @@
         <v>775</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1100</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>0.419</v>
+        <v>2000</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>1.580645161290323</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -929,7 +940,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Optic Choice parallel rookie auto PSA 10; base Optic auto PSA 10 ~$500-800, Choice premium</t>
+          <t>Choice parallel auto PSA 10 scarce; Opti-Graphs Choice PSA 10/10 ~$600; Rated Rookie auto Choice more desirable</t>
         </is>
       </c>
     </row>
@@ -951,14 +962,14 @@
         <v>860</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>0.395</v>
+        <v>2500</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>1.906976744186047</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -968,7 +979,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Flawless Ruby /15 draft gem insert; Ant premium cards trending up</t>
+          <t>Flawless Momentous Autos Ruby /15 last sold raw $3,650; Draft Gem Sigs Ruby /15 comparable</t>
         </is>
       </c>
     </row>
@@ -990,10 +1001,10 @@
         <v>860</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7440000000000001</v>
+        <v>1.906976744186047</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -1002,12 +1013,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Med-High</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Dual jersey Kobe+MJ iconic pairing; BGS 8.5 mid-grade; comparable duals $1,000-2,000</t>
+          <t>2004-05 SP Game Used Auth Dual Patch /25 BGS 8.5 sold $2,773; iconic Kobe+MJ pairing</t>
         </is>
       </c>
     </row>
@@ -1068,14 +1079,14 @@
         <v>362</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>800</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>STRONG BUY</t>
+        <v>400</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>0.1049723756906077</v>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>FAIR</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1085,7 +1096,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Courtside Gold /10 premium parallel; PSA 9 Luka low-number cards $600-1,000</t>
+          <t>2023 Select Courtside Gold Disco /10 PSA 10 sold $516 Fanatics; PSA 9 discount; non-rookie year</t>
         </is>
       </c>
     </row>
@@ -1107,24 +1118,24 @@
         <v>680</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0.765</v>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>STRONG BUY</t>
+        <v>500</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>-0.2647058823529412</v>
+      </c>
+      <c r="G15" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Iverson Prizm Black Gold PSA 10 pop 2 with jersey match; legacy player premium</t>
+          <t>Iverson Prizm Deca Gold /10 raw sold $195; PSA 10 pop 2 + jersey match premium; HOF but soft market</t>
         </is>
       </c>
     </row>
@@ -1146,14 +1157,14 @@
         <v>600</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>STRONG BUY</t>
+        <v>500</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>-0.1666666666666667</v>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1163,7 +1174,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>SGA NT Emerald /5 ultra-low numbered; SGA MVP-caliber demand; Viewpoint subset</t>
+          <t>2024-25 NT Viewpoint Sigs Emerald listed $475; SGA MVP surge; secondary insert not flagship RPA</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1199,7 @@
         <v>1200</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>1.667</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
@@ -1197,12 +1208,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Gold patch auto /10 of current MVP candidate; Immaculate premium product</t>
+          <t>2021 Immaculate SGA Patch Auto Gold /10 sold ~C$1,378 (~$1K USD) PSA Auto 9; market hotter post-MVP</t>
         </is>
       </c>
     </row>
@@ -1224,10 +1235,10 @@
         <v>450</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.778</v>
+        <v>2.333333333333333</v>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
@@ -1236,12 +1247,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>NT-style patch auto /15; Curry autos in premium products consistently $500-1,000</t>
+          <t>Curry patch autos premium sets /15-25 range $1,500-5,000; Regalia secondary insert; splitting range</t>
         </is>
       </c>
     </row>
@@ -1263,10 +1274,10 @@
         <v>285</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.754</v>
+        <v>1.807017543859649</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
@@ -1275,12 +1286,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Flawless USA Basketball /10; KD premium but not auto; $400-600 range</t>
+          <t>KD Flawless /10 no auto typically $500-1,200; USA Basketball niche appeal</t>
         </is>
       </c>
     </row>
@@ -1302,14 +1313,14 @@
         <v>585</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>800</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>0.368</v>
+        <v>1200</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>1.051282051282051</v>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1319,7 +1330,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Topps Mercury Gold Refractor /50 PSA 10; Fanatics Collect listing found Oct 2025 sale</t>
+          <t>Listed on Fanatics Collect sold Oct 2025; PSA pop 1 of 3; non-auto gold /50 Wemby RC</t>
         </is>
       </c>
     </row>
@@ -1341,14 +1352,14 @@
         <v>610</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>900</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>0.475</v>
+        <v>1200</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0.9672131147540983</v>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1358,7 +1369,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Bowman U Red /10 auto; CC cards volatile but strong demand; PSA 9</t>
+          <t>Goldin Nov 2024 sold Red #26B Auto graded 9 for $1,159; Bowman U Best Red /10 similar range</t>
         </is>
       </c>
     </row>
@@ -1380,14 +1391,14 @@
         <v>235</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>400</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>0.7020000000000001</v>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>STRONG BUY</t>
+        <v>250</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>0.06382978723404255</v>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>FAIR</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1397,7 +1408,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>One and One Blue /49; Jokic 3x MVP; non-auto but low-numbered</t>
+          <t>One &amp; One Blue /49 non-auto; Timeless Moments Auto /99 sold $750 raw; non-auto drops to $150-300</t>
         </is>
       </c>
     </row>
@@ -1419,24 +1430,24 @@
         <v>575</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>800</v>
-      </c>
-      <c r="F23" s="7" t="n">
-        <v>0.391</v>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>300</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>-0.4782608695652174</v>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Low-Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Yao auto /25 in Gold Standard; HOF player; Mother Lode patch auto premium</t>
+          <t>Yao autos premium sets $150-500; Gold Standard Mother Lode niche 2012-13 product; comparable HOF autos $100-200</t>
         </is>
       </c>
     </row>
@@ -1458,10 +1469,10 @@
         <v>415</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.6870000000000001</v>
+        <v>1.409638554216867</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
@@ -1470,12 +1481,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Contenders Optic Orange /15 PSA 10 w/10 auto; Tatum top player; premium parallel</t>
+          <t>Contenders Optic '85 Tribute Green /49 PSA 10 guide $1,000; Orange /15 scarcer; post-championship Tatum</t>
         </is>
       </c>
     </row>
@@ -1497,24 +1508,24 @@
         <v>475</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>600</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>0.263</v>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>300</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>-0.3684210526315789</v>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Court Kings All Kings insert PSA 9; Giannis premium insert</t>
+          <t>Court Kings insert non-auto non-numbered; Giannis inserts PSA 9 typically $50-250; splitting high</t>
         </is>
       </c>
     </row>
@@ -1536,10 +1547,10 @@
         <v>340</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.765</v>
+        <v>1.941176470588235</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
@@ -1548,12 +1559,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Select Tie-Dye /25 BGS 9.5 w/10 auto; popular parallel</t>
+          <t>Select Tie-Dye /25 BGS 9.5/10; if auto value much higher; non-rookie year but premium parallel</t>
         </is>
       </c>
     </row>
@@ -1575,10 +1586,10 @@
         <v>160</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>350</v>
+        <v>1500</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>1.188</v>
+        <v>8.375</v>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
@@ -1587,12 +1598,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>One and One /25 BGS 9 w/10 auto; pop 3; Curry premium</t>
+          <t>Curry One &amp; One Black Color Blast sold $678 raw; /25 auto BGS 9/10 pop 3 premium; evergreen demand</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3081,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Tier C FMV estimates with research-backed values
Major findings: Luka Spectra Neon Pink /25 PSA 9 is a rookie auto
worth ~$3K (at $145 bid), Ant Optic Fast Break Gold /10 ~$3.5K (at
$250 bid), Ant NT Private Signings ~$2.5K (at $211). LeBron eTopps
PSA 9 actually overpriced at $231 (FMV ~$200, high confidence).
Total FMV now $72,790 vs $25,060 bids (191% upside).

https://claude.ai/code/session_01GTThiDtMm869wgd52PwWVn
</commit_message>
<xml_diff>
--- a/Inventory/Goldin_Auction_FMV.xlsx
+++ b/Inventory/Goldin_Auction_FMV.xlsx
@@ -1625,14 +1625,14 @@
         <v>510</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>700</v>
-      </c>
-      <c r="F28" s="7" t="n">
-        <v>0.373</v>
+        <v>2000</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>2.92156862745098</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>PSA 9 sold ~$2,375 in 2021; market corrected since; current ~$600-800</t>
+          <t>PSA 9 sold $2,375 (Nov 2021); market softened but Luka NT autos still command premium</t>
         </is>
       </c>
     </row>
@@ -1664,24 +1664,24 @@
         <v>515</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>700</v>
-      </c>
-      <c r="F29" s="7" t="n">
-        <v>0.359</v>
+        <v>1200</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>1.330097087378641</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Immaculate Scorers Club insert /25; Luka auto premium</t>
+          <t>Immaculate non-RPA Luka autos /25 trade below NT; estimated from NT Treasured Sigs discount</t>
         </is>
       </c>
     </row>
@@ -1703,10 +1703,10 @@
         <v>211</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>400</v>
+        <v>2500</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.8959999999999999</v>
+        <v>10.84834123222749</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>NT Private Signings auto; pop 4; Ant premium</t>
+          <t>Raw Private Signings listed $1,500-2,500 eBay; non-patch auto but low pop 4 scarcity premium</t>
         </is>
       </c>
     </row>
@@ -1742,10 +1742,10 @@
         <v>250</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>500</v>
+        <v>3500</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Optic Fast Break Gold /10 PSA 9 pop 3; scarce parallel</t>
+          <t>Fast Break Gold scarce retail-exclusive; Mosaic FB Gold /10 PSA 10 ~$4K+; PSA 9 pop 3 rookie auto</t>
         </is>
       </c>
     </row>
@@ -1781,10 +1781,10 @@
         <v>325</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.5379999999999999</v>
+        <v>3.615384615384615</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>1/1 BGS 10 Pristine w/10 auto; Linsanity nostalgia; niche player but perfect grade 1/1</t>
+          <t>1/1 BGS 10 Pristine w/10 auto exceptional; Linsanity nostalgia; niche but perfect grade</t>
         </is>
       </c>
     </row>
@@ -1820,10 +1820,10 @@
         <v>155</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>300</v>
+        <v>1500</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.9350000000000001</v>
+        <v>8.67741935483871</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Five Star /30 first serial; Sasaki MLB buzz; #01/30 jersey number premium</t>
+          <t>Sasaki Chrome Logofractor Gold Auto /50 sold $984; Five Star premium; #01/30 first serial premium</t>
         </is>
       </c>
     </row>
@@ -1859,14 +1859,14 @@
         <v>231</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>350</v>
-      </c>
-      <c r="F34" s="5" t="n">
-        <v>0.515</v>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>STRONG BUY</t>
+        <v>200</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>-0.1341991341991342</v>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>2003 eTopps RC PSA 9; well-tracked card; recent sales $300-400</t>
+          <t>Multiple PSA 9 sales 2025: $202, $217, $221, $231, $150; clear market $150-230</t>
         </is>
       </c>
     </row>
@@ -1898,14 +1898,14 @@
         <v>265</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>350</v>
-      </c>
-      <c r="F35" s="7" t="n">
-        <v>0.321</v>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>300</v>
+      </c>
+      <c r="F35" s="17" t="n">
+        <v>0.1320754716981132</v>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>FAIR</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Downtown insert PSA 10; WNBA growing market</t>
+          <t>Downtown marquee Donruss insert; WNBA star; PSA 10 Downtown for stars $200-500</t>
         </is>
       </c>
     </row>
@@ -1937,10 +1937,10 @@
         <v>120</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>250</v>
+        <v>800</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>1.083</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Flawless Excellence 1/1 auto; Chet upside but injury concerns</t>
+          <t>Chet Flawless autos /25 range $200-500; 1/1 adds 2-3x premium despite injury concerns</t>
         </is>
       </c>
     </row>
@@ -1976,10 +1976,10 @@
         <v>80</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.875</v>
+        <v>5.25</v>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
@@ -1988,12 +1988,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Eminence Gold /5 auto; low-numbered Chet auto</t>
+          <t>Eminence premium Panini product; /5 Gold auto scarce; based on Flawless /10-25 autos $150-350</t>
         </is>
       </c>
     </row>
@@ -2015,10 +2015,10 @@
         <v>160</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>300</v>
+        <v>1500</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.875</v>
+        <v>8.375</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Exquisite /30 BGS 9 w/10 auto; HOF player; premium product</t>
+          <t>Carter Exquisite iconic 2000s; BGS 9/10 strong grade; HOF induction boosted market; $1K-2.5K range</t>
         </is>
       </c>
     </row>
@@ -2054,10 +2054,10 @@
         <v>152</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.645</v>
+        <v>1.631578947368421</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Flawless Gold /10 BGS 8; legend but mid-grade</t>
+          <t>Erving Flawless 1/1 autos sold $325-450; Gold /10 non-auto BGS 8 less desirable</t>
         </is>
       </c>
     </row>
@@ -2093,10 +2093,10 @@
         <v>121</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.653</v>
+        <v>1.892561983471074</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Exquisite Sigs /30 PSA 9; Dr. J auto</t>
+          <t>Exquisite Sigs desirable for HOFers; /30 PSA 9 solid; vintage legend autos $250-500</t>
         </is>
       </c>
     </row>
@@ -2132,10 +2132,10 @@
         <v>198</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>350</v>
+        <v>500</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.768</v>
+        <v>1.525252525252525</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Triple jersey w/ Kobe+LeBron+Oscar; iconic combo; BGS 8 mid-grade</t>
+          <t>SP Game Used triple swatch; Kobe+LeBron combo highly collectible; BGS 8 lower grade</t>
         </is>
       </c>
     </row>
@@ -2171,10 +2171,10 @@
         <v>102</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.961</v>
+        <v>2.92156862745098</v>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Immaculate Red patch auto /15; AD steady market</t>
+          <t>AD Immaculate Sneaker Swatches Sigs /15 listed $367 COMC; Red patch auto comparable</t>
         </is>
       </c>
     </row>
@@ -2210,14 +2210,14 @@
         <v>228</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>300</v>
-      </c>
-      <c r="F43" s="7" t="n">
-        <v>0.316</v>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>200</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>-0.1228070175438596</v>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Absolute 3 swatch /199 PSA 8 pop 2; Maxey rising star</t>
+          <t>Maxey surged 150%+; Absolute 3 Swatch /199 mid-tier rookie mem; PSA 8 lower but pop 2</t>
         </is>
       </c>
     </row>
@@ -2249,10 +2249,10 @@
         <v>145</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.7240000000000001</v>
+        <v>3.137931034482758</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -2261,12 +2261,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Crown Royale Silhouette Gold /10; premium parallel</t>
+          <t>Crown Royale Silhouette popular die-cut; Gold /10 very scarce; Maxey rising star</t>
         </is>
       </c>
     </row>
@@ -2288,24 +2288,24 @@
         <v>215</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>275</v>
-      </c>
-      <c r="F45" s="7" t="n">
-        <v>0.279</v>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>150</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>-0.3023255813953488</v>
+      </c>
+      <c r="G45" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Flawless Vault memorabilia /25 PSA 8; KAT steady</t>
+          <t>KAT Flawless /25 listed $100-200 eBay; non-auto mem PSA 8 modest; moderate market</t>
         </is>
       </c>
     </row>
@@ -2327,24 +2327,24 @@
         <v>161</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="F46" s="5" t="n">
-        <v>0.5529999999999999</v>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>STRONG BUY</t>
+        <v>150</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>-0.06832298136645963</v>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Select Red Cracked Ice PSA 10; Wemby base parallel</t>
+          <t>Premier Level Red Cracked Ice PSA 10 sold $128.75 (Jan 2025); Blue $62-99; Red ~$125-175</t>
         </is>
       </c>
     </row>
@@ -2366,10 +2366,10 @@
         <v>145</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>250</v>
+        <v>3000</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.7240000000000001</v>
+        <v>19.68965517241379</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Spectra Neon Pink /25 PSA 9; popular Luka parallel</t>
+          <t>2018-19 Spectra Neon Pink Jersey Auto RC /25 PSA 9; one of best Spectra parallels; peak discounted</t>
         </is>
       </c>
     </row>
@@ -2405,10 +2405,10 @@
         <v>155</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>350</v>
+        <v>800</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>1.258</v>
+        <v>4.161290322580645</v>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Flawless Premium Ink auto /25 BGS 9.5 w/10; Giannis auto premium</t>
+          <t>Flawless Momentous Jersey Patch Auto /25 BGS 9.5 sold $790; Premium Ink comparable auto subset</t>
         </is>
       </c>
     </row>
@@ -2444,10 +2444,10 @@
         <v>130</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0.5379999999999999</v>
+        <v>1.307692307692308</v>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
@@ -2456,12 +2456,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Obsidian Matrix Yellow /10; low-numbered Giannis</t>
+          <t>Obsidian mid-tier product; Yellow /10 scarce but doesn't command Flawless/NT premiums</t>
         </is>
       </c>
     </row>
@@ -2483,14 +2483,14 @@
         <v>160</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="F50" s="5" t="n">
-        <v>0.5620000000000001</v>
+        <v>200</v>
+      </c>
+      <c r="F50" s="17" t="n">
+        <v>0.25</v>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Topps NPB Chrome Orange /25; Japanese baseball star</t>
+          <t>2021 Topps Chrome NPB '86 Orange /25 PSA 9 sold ~$180; MLB transition hype but pre-MLB product</t>
         </is>
       </c>
     </row>
@@ -2522,10 +2522,10 @@
         <v>67</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>0.7909999999999999</v>
+        <v>3.477611940298508</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>All-Time Greats /50 BGS 9.5; legend non-auto</t>
+          <t>Legend non-auto /50 BGS 9.5; ATG or similar; legend autos premium products $200-500</t>
         </is>
       </c>
     </row>
@@ -2561,10 +2561,10 @@
         <v>14</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>2.571</v>
+        <v>34.71428571428572</v>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>VIP Gold mem /5 BGS 8; low-grade niche</t>
+          <t>Panini VIP Gold /5 extremely scarce convention exclusive; Curry premium; BGS 8 lower grade</t>
         </is>
       </c>
     </row>
@@ -2600,10 +2600,10 @@
         <v>30</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>60</v>
+        <v>250</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>1</v>
+        <v>7.333333333333333</v>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>VIP Cracked Ice /50; convention exclusive</t>
+          <t>Panini VIP Cracked Ice /50 convention cards; BGS 9.5 strong; 2016 VIP Cracked Ice listed on eBay</t>
         </is>
       </c>
     </row>
@@ -2639,14 +2639,14 @@
         <v>105</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="F54" s="7" t="n">
-        <v>0.429</v>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>75</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>-0.2857142857142857</v>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Prizm Swatches Orange Ice; BGS Authentic (ungraded card)</t>
+          <t>Curry Prizm Sensational Swatches base raw $38; Orange Ice scarcer BUT BGS Auth = trimmed/altered, hurts value</t>
         </is>
       </c>
     </row>
@@ -2678,14 +2678,14 @@
         <v>42</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="F55" s="7" t="n">
-        <v>0.429</v>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>50</v>
+      </c>
+      <c r="F55" s="17" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>FAIR</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Prestige True Colors; lower-tier product</t>
+          <t>Prestige True Colors jersey insert budget product; BGS 9; lower-tier Curry mem $30-75</t>
         </is>
       </c>
     </row>
@@ -2717,10 +2717,10 @@
         <v>10</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Immaculate Ink auto /25 PSA 8; Ray Allen HOF</t>
+          <t>Immaculate Ink Red /25 auto listed ~$204 COMC; PSA 8 discount; Ray Allen HOF steady demand</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update all 62 cards to conservative sell-comfortable FMV values
Revised down across the board to prices the user would be comfortable
selling at. Total FMV $55,695 vs $25,060 bids (122% upside).
44 STRONG BUY, 1 BUY, 5 FAIR, 12 HOLD/PASS.

https://claude.ai/code/session_01GTThiDtMm869wgd52PwWVn
</commit_message>
<xml_diff>
--- a/Inventory/Goldin_Auction_FMV.xlsx
+++ b/Inventory/Goldin_Auction_FMV.xlsx
@@ -611,10 +611,10 @@
         <v>1588</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>1.519</v>
+        <v>0.889168765743073</v>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
@@ -623,12 +623,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>1/1 NT patch auto; Shaq autos /25 sell $1-3K, 1/1 premium</t>
+          <t>No comp; 1/1 Shaq NT autos range wide</t>
         </is>
       </c>
     </row>
@@ -650,10 +650,10 @@
         <v>1051</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1250</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>0.189</v>
+        <v>1200</v>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>0.1417697431018078</v>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
@@ -662,12 +662,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Recent PSA 8 sales: $2,275 (Nov), $1,275 (Oct), $1,199 (Oct 2025)</t>
+          <t>Sold $1,199-$2,275 recent; safe at $1,200</t>
         </is>
       </c>
     </row>
@@ -689,10 +689,10 @@
         <v>1400</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>6000</v>
+        <v>4000</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>3.286</v>
+        <v>1.857142857142857</v>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
@@ -701,12 +701,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Prizm Deca Gold /10 Curry sold $7,320 Goldin; Kaleidoscopic Gold /10 PSA 10 ultra rare</t>
+          <t>No direct comp; Deca Gold /10 sold $7,320</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
         <v>1400</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>-0.001</v>
+        <v>-0.0007137758743754461</v>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
@@ -740,12 +740,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Med-High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>PSA 10 sold $1,424 (Jun 2025 per PSA auction prices)</t>
+          <t>PSA data: sold $1,424</t>
         </is>
       </c>
     </row>
@@ -767,24 +767,24 @@
         <v>1512</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>0.323</v>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>1800</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>FAIR</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Purple /35 listed $2,200; PSA Auth discounted vs graded; /35 blue RPA</t>
+          <t>PSA Auth hurts value; Purple /35 listed $2,200</t>
         </is>
       </c>
     </row>
@@ -806,10 +806,10 @@
         <v>1601</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>3.997</v>
+        <v>2.123048094940662</v>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
@@ -818,12 +818,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Modern mfg relic but iconic trio; pop 2 PSA 10; comparable legend relics $5-12K</t>
+          <t>Modern relic; iconic names; wide range $3-10K</t>
         </is>
       </c>
     </row>
@@ -845,10 +845,10 @@
         <v>803</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>2.113</v>
+        <v>1.4906600249066</v>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
@@ -857,12 +857,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>NT Clutch Factor Jersey Sigs /25 BGS 9.5 listed $2,500; PSA 9 slight discount</t>
+          <t>BGS 9.5 listed $2,500; PSA 9 discount</t>
         </is>
       </c>
     </row>
@@ -884,24 +884,24 @@
         <v>910</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.6483516483516484</v>
+        <v>1200</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>0.3186813186813187</v>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Base prospect auto raw sold $1,000 (Dec 2025); PSA 10 premium; Superfractor 1/1 PSA 10 sold $18K</t>
+          <t>Raw sold $1K Dec 2025; PSA 10 bump</t>
         </is>
       </c>
     </row>
@@ -923,10 +923,10 @@
         <v>775</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>1.580645161290323</v>
+        <v>0.9354838709677419</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
@@ -935,12 +935,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Choice parallel auto PSA 10 scarce; Opti-Graphs Choice PSA 10/10 ~$600; Rated Rookie auto Choice more desirable</t>
+          <t>Choice scarce; base Optic auto ~$600</t>
         </is>
       </c>
     </row>
@@ -962,10 +962,10 @@
         <v>860</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1.906976744186047</v>
+        <v>1.325581395348837</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -974,12 +974,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Flawless Momentous Autos Ruby /15 last sold raw $3,650; Draft Gem Sigs Ruby /15 comparable</t>
+          <t>Ruby /15 raw sold $3,650; conservative</t>
         </is>
       </c>
     </row>
@@ -1001,10 +1001,10 @@
         <v>860</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>1.906976744186047</v>
+        <v>1.325581395348837</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Med-High</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2004-05 SP Game Used Auth Dual Patch /25 BGS 8.5 sold $2,773; iconic Kobe+MJ pairing</t>
+          <t>Dual Patch /25 BGS 8.5 sold $2,773</t>
         </is>
       </c>
     </row>
@@ -1040,10 +1040,10 @@
         <v>810</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>1.469</v>
+        <v>0.8518518518518519</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Prizm Mojo auto /25 is premium; Luka autos in low-number Prizm consistently $1,500+</t>
+          <t>Year matters hugely; if not RC then ~$1-2K</t>
         </is>
       </c>
     </row>
@@ -1091,12 +1091,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2023 Select Courtside Gold Disco /10 PSA 10 sold $516 Fanatics; PSA 9 discount; non-rookie year</t>
+          <t>Gold Disco /10 PSA 10 sold $516; PSA 9 less</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1130,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Iverson Prizm Deca Gold /10 raw sold $195; PSA 10 pop 2 + jersey match premium; HOF but soft market</t>
+          <t>Deca Gold /10 raw $195; PSA 10 pop 2 premium</t>
         </is>
       </c>
     </row>
@@ -1157,10 +1157,10 @@
         <v>600</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>500</v>
+        <v>475</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>-0.1666666666666667</v>
+        <v>-0.2083333333333333</v>
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
@@ -1169,12 +1169,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2024-25 NT Viewpoint Sigs Emerald listed $475; SGA MVP surge; secondary insert not flagship RPA</t>
+          <t>Listed $475; secondary insert not RPA</t>
         </is>
       </c>
     </row>
@@ -1196,10 +1196,10 @@
         <v>450</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>1.666666666666667</v>
+        <v>1.222222222222222</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
@@ -1208,12 +1208,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2021 Immaculate SGA Patch Auto Gold /10 sold ~C$1,378 (~$1K USD) PSA Auto 9; market hotter post-MVP</t>
+          <t>SGA Patch Auto Gold /10 sold ~$1K CAD</t>
         </is>
       </c>
     </row>
@@ -1235,10 +1235,10 @@
         <v>450</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>2.333333333333333</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
@@ -1247,12 +1247,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Curry patch autos premium sets /15-25 range $1,500-5,000; Regalia secondary insert; splitting range</t>
+          <t>Curry patch autos /15 range $1-3K</t>
         </is>
       </c>
     </row>
@@ -1274,10 +1274,10 @@
         <v>285</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1.807017543859649</v>
+        <v>1.105263157894737</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
@@ -1286,12 +1286,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>KD Flawless /10 no auto typically $500-1,200; USA Basketball niche appeal</t>
+          <t>No auto; KD Flawless /10 $500-1,200</t>
         </is>
       </c>
     </row>
@@ -1313,10 +1313,10 @@
         <v>585</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>1.051282051282051</v>
+        <v>0.7094017094017094</v>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
@@ -1325,12 +1325,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Listed on Fanatics Collect sold Oct 2025; PSA pop 1 of 3; non-auto gold /50 Wemby RC</t>
+          <t>Fanatics sold Oct 2025; pop 1 of 3</t>
         </is>
       </c>
     </row>
@@ -1352,10 +1352,10 @@
         <v>610</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.9672131147540983</v>
+        <v>0.8032786885245902</v>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Goldin Nov 2024 sold Red #26B Auto graded 9 for $1,159; Bowman U Best Red /10 similar range</t>
+          <t>Goldin sold $1,159 Nov 2024 same card</t>
         </is>
       </c>
     </row>
@@ -1391,24 +1391,24 @@
         <v>235</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="F22" s="17" t="n">
-        <v>0.06382978723404255</v>
+        <v>200</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>-0.148936170212766</v>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>FAIR</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>One &amp; One Blue /49 non-auto; Timeless Moments Auto /99 sold $750 raw; non-auto drops to $150-300</t>
+          <t>Non-auto; /49 base parallel</t>
         </is>
       </c>
     </row>
@@ -1430,10 +1430,10 @@
         <v>575</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>-0.4782608695652174</v>
+        <v>-0.5652173913043478</v>
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
@@ -1442,12 +1442,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Yao autos premium sets $150-500; Gold Standard Mother Lode niche 2012-13 product; comparable HOF autos $100-200</t>
+          <t>Niche 2012-13 product; comparable HOF $100-200</t>
         </is>
       </c>
     </row>
@@ -1469,10 +1469,10 @@
         <v>415</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>1.409638554216867</v>
+        <v>0.927710843373494</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Contenders Optic '85 Tribute Green /49 PSA 10 guide $1,000; Orange /15 scarcer; post-championship Tatum</t>
+          <t>Green /49 PSA 10 guide $1K; Orange /15 scarcer</t>
         </is>
       </c>
     </row>
@@ -1508,10 +1508,10 @@
         <v>475</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>-0.3684210526315789</v>
+        <v>-0.5789473684210527</v>
       </c>
       <c r="G25" s="18" t="inlineStr">
         <is>
@@ -1520,12 +1520,12 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Court Kings insert non-auto non-numbered; Giannis inserts PSA 9 typically $50-250; splitting high</t>
+          <t>Non-auto non-numbered insert</t>
         </is>
       </c>
     </row>
@@ -1547,10 +1547,10 @@
         <v>340</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>1.941176470588235</v>
+        <v>1.352941176470588</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Select Tie-Dye /25 BGS 9.5/10; if auto value much higher; non-rookie year but premium parallel</t>
+          <t>Need to know if auto; if not, much less</t>
         </is>
       </c>
     </row>
@@ -1586,10 +1586,10 @@
         <v>160</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>8.375</v>
+        <v>6.5</v>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
@@ -1598,12 +1598,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Curry One &amp; One Black Color Blast sold $678 raw; /25 auto BGS 9/10 pop 3 premium; evergreen demand</t>
+          <t>Color Blast sold $678 raw; /25 auto premium</t>
         </is>
       </c>
     </row>
@@ -1625,10 +1625,10 @@
         <v>510</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>2.92156862745098</v>
+        <v>1.941176470588235</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
@@ -1637,12 +1637,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>PSA 9 sold $2,375 (Nov 2021); market softened but Luka NT autos still command premium</t>
+          <t>Sold $2,375 in 2021; market down 30-40%</t>
         </is>
       </c>
     </row>
@@ -1664,10 +1664,10 @@
         <v>515</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>1.330097087378641</v>
+        <v>0.7475728155339806</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Immaculate non-RPA Luka autos /25 trade below NT; estimated from NT Treasured Sigs discount</t>
+          <t>Below NT equivalent; Luka auto /25</t>
         </is>
       </c>
     </row>
@@ -1703,10 +1703,10 @@
         <v>211</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>10.84834123222749</v>
+        <v>7.530805687203792</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
@@ -1715,12 +1715,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Raw Private Signings listed $1,500-2,500 eBay; non-patch auto but low pop 4 scarcity premium</t>
+          <t>Listed $1,500-2,500; non-patch auto</t>
         </is>
       </c>
     </row>
@@ -1742,10 +1742,10 @@
         <v>250</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Fast Break Gold scarce retail-exclusive; Mosaic FB Gold /10 PSA 10 ~$4K+; PSA 9 pop 3 rookie auto</t>
+          <t>FB Gold retail-exclusive scarce; pop 3</t>
         </is>
       </c>
     </row>
@@ -1781,10 +1781,10 @@
         <v>325</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>3.615384615384615</v>
+        <v>2.076923076923077</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1793,12 +1793,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>1/1 BGS 10 Pristine w/10 auto exceptional; Linsanity nostalgia; niche but perfect grade</t>
+          <t>No comp; 1/1 + BGS 10 Pristine but niche player</t>
         </is>
       </c>
     </row>
@@ -1820,10 +1820,10 @@
         <v>155</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>8.67741935483871</v>
+        <v>6.741935483870968</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
@@ -1832,12 +1832,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Sasaki Chrome Logofractor Gold Auto /50 sold $984; Five Star premium; #01/30 first serial premium</t>
+          <t>Chrome Auto /50 sold $984; Five Star + #01 premium</t>
         </is>
       </c>
     </row>
@@ -1871,12 +1871,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Multiple PSA 9 sales 2025: $202, $217, $221, $231, $150; clear market $150-230</t>
+          <t>Sold $150-$231 multiple times 2025</t>
         </is>
       </c>
     </row>
@@ -1898,10 +1898,10 @@
         <v>265</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>300</v>
+        <v>275</v>
       </c>
       <c r="F35" s="17" t="n">
-        <v>0.1320754716981132</v>
+        <v>0.03773584905660377</v>
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
@@ -1910,12 +1910,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Downtown marquee Donruss insert; WNBA star; PSA 10 Downtown for stars $200-500</t>
+          <t>Downtown insert WNBA star</t>
         </is>
       </c>
     </row>
@@ -1937,10 +1937,10 @@
         <v>120</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>5.666666666666667</v>
+        <v>4</v>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
@@ -1949,12 +1949,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Chet Flawless autos /25 range $200-500; 1/1 adds 2-3x premium despite injury concerns</t>
+          <t>Chet cooled; 1/1 auto still scarce</t>
         </is>
       </c>
     </row>
@@ -1976,10 +1976,10 @@
         <v>80</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>5.25</v>
+        <v>4</v>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
@@ -1988,12 +1988,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Eminence premium Panini product; /5 Gold auto scarce; based on Flawless /10-25 autos $150-350</t>
+          <t>/5 auto premium but Chet soft</t>
         </is>
       </c>
     </row>
@@ -2015,10 +2015,10 @@
         <v>160</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>8.375</v>
+        <v>6.5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -2027,12 +2027,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Carter Exquisite iconic 2000s; BGS 9/10 strong grade; HOF induction boosted market; $1K-2.5K range</t>
+          <t>HOF; Exquisite iconic; BGS 9/10 solid</t>
         </is>
       </c>
     </row>
@@ -2054,10 +2054,10 @@
         <v>152</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>1.631578947368421</v>
+        <v>1.302631578947368</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Erving Flawless 1/1 autos sold $325-450; Gold /10 non-auto BGS 8 less desirable</t>
+          <t>1/1 autos sold $325-450; Gold /10 less</t>
         </is>
       </c>
     </row>
@@ -2093,10 +2093,10 @@
         <v>121</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>1.892561983471074</v>
+        <v>1.479338842975207</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Exquisite Sigs desirable for HOFers; /30 PSA 9 solid; vintage legend autos $250-500</t>
+          <t>Legend Exquisite autos $250-500</t>
         </is>
       </c>
     </row>
@@ -2132,10 +2132,10 @@
         <v>198</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>1.525252525252525</v>
+        <v>1.02020202020202</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>SP Game Used triple swatch; Kobe+LeBron combo highly collectible; BGS 8 lower grade</t>
+          <t>Iconic combo but BGS 8 mid-grade</t>
         </is>
       </c>
     </row>
@@ -2171,10 +2171,10 @@
         <v>102</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>2.92156862745098</v>
+        <v>2.431372549019608</v>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
@@ -2183,12 +2183,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>AD Immaculate Sneaker Swatches Sigs /15 listed $367 COMC; Red patch auto comparable</t>
+          <t>Sneaker Swatches Sigs /15 listed $367</t>
         </is>
       </c>
     </row>
@@ -2210,24 +2210,24 @@
         <v>228</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="F43" s="9" t="n">
-        <v>-0.1228070175438596</v>
-      </c>
-      <c r="G43" s="8" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>-0.2324561403508772</v>
+      </c>
+      <c r="G43" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Maxey surged 150%+; Absolute 3 Swatch /199 mid-tier rookie mem; PSA 8 lower but pop 2</t>
+          <t>Mid-tier mem card; pop 2 helps</t>
         </is>
       </c>
     </row>
@@ -2249,10 +2249,10 @@
         <v>145</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>3.137931034482758</v>
+        <v>2.103448275862069</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -2261,12 +2261,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Crown Royale Silhouette popular die-cut; Gold /10 very scarce; Maxey rising star</t>
+          <t>Silhouette popular; Gold /10 scarce</t>
         </is>
       </c>
     </row>
@@ -2288,10 +2288,10 @@
         <v>215</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="F45" s="9" t="n">
-        <v>-0.3023255813953488</v>
+        <v>-0.4186046511627907</v>
       </c>
       <c r="G45" s="18" t="inlineStr">
         <is>
@@ -2300,12 +2300,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>KAT Flawless /25 listed $100-200 eBay; non-auto mem PSA 8 modest; moderate market</t>
+          <t>Non-auto mem; KAT moderate market</t>
         </is>
       </c>
     </row>
@@ -2327,24 +2327,24 @@
         <v>161</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>-0.06832298136645963</v>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>-0.1925465838509317</v>
+      </c>
+      <c r="G46" s="18" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Premier Level Red Cracked Ice PSA 10 sold $128.75 (Jan 2025); Blue $62-99; Red ~$125-175</t>
+          <t>Sold $129 Jan 2025</t>
         </is>
       </c>
     </row>
@@ -2366,10 +2366,10 @@
         <v>145</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>19.68965517241379</v>
+        <v>12.79310344827586</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -2378,12 +2378,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>2018-19 Spectra Neon Pink Jersey Auto RC /25 PSA 9; one of best Spectra parallels; peak discounted</t>
+          <t>IF RC auto=$3K; if later year=$300. VERIFY YEAR</t>
         </is>
       </c>
     </row>
@@ -2405,10 +2405,10 @@
         <v>155</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>4.161290322580645</v>
+        <v>3.516129032258065</v>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
@@ -2417,12 +2417,12 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Flawless Momentous Jersey Patch Auto /25 BGS 9.5 sold $790; Premium Ink comparable auto subset</t>
+          <t>Momentous Patch Auto /25 BGS 9.5 sold $790</t>
         </is>
       </c>
     </row>
@@ -2444,10 +2444,10 @@
         <v>130</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>1.307692307692308</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
@@ -2456,12 +2456,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Obsidian mid-tier product; Yellow /10 scarce but doesn't command Flawless/NT premiums</t>
+          <t>Mid-tier product; /10 scarce</t>
         </is>
       </c>
     </row>
@@ -2483,24 +2483,24 @@
         <v>160</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="F50" s="17" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>0.125</v>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>FAIR</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>2021 Topps Chrome NPB '86 Orange /25 PSA 9 sold ~$180; MLB transition hype but pre-MLB product</t>
+          <t>NPB Chrome '86 Orange /25 sold ~$180</t>
         </is>
       </c>
     </row>
@@ -2522,10 +2522,10 @@
         <v>67</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>3.477611940298508</v>
+        <v>2.73134328358209</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Legend non-auto /50 BGS 9.5; ATG or similar; legend autos premium products $200-500</t>
+          <t>Legend non-auto /50</t>
         </is>
       </c>
     </row>
@@ -2561,10 +2561,10 @@
         <v>14</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>34.71428571428572</v>
+        <v>27.57142857142857</v>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Panini VIP Gold /5 extremely scarce convention exclusive; Curry premium; BGS 8 lower grade</t>
+          <t>/5 convention exclusive; BGS 8 hurts</t>
         </is>
       </c>
     </row>
@@ -2600,10 +2600,10 @@
         <v>30</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>7.333333333333333</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
@@ -2612,12 +2612,12 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Panini VIP Cracked Ice /50 convention cards; BGS 9.5 strong; 2016 VIP Cracked Ice listed on eBay</t>
+          <t>Convention niche</t>
         </is>
       </c>
     </row>
@@ -2639,10 +2639,10 @@
         <v>105</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>-0.2857142857142857</v>
+        <v>-0.4285714285714285</v>
       </c>
       <c r="G54" s="18" t="inlineStr">
         <is>
@@ -2651,12 +2651,12 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Curry Prizm Sensational Swatches base raw $38; Orange Ice scarcer BUT BGS Auth = trimmed/altered, hurts value</t>
+          <t>BGS Auth = trimmed/altered. Damaged goods</t>
         </is>
       </c>
     </row>
@@ -2678,24 +2678,24 @@
         <v>42</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F55" s="17" t="n">
-        <v>0.1904761904761905</v>
+        <v>40</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>-0.04761904761904762</v>
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>FAIR</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Prestige True Colors jersey insert budget product; BGS 9; lower-tier Curry mem $30-75</t>
+          <t>Budget product jersey insert</t>
         </is>
       </c>
     </row>
@@ -2717,10 +2717,10 @@
         <v>10</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>14</v>
+        <v>11.5</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Immaculate Ink Red /25 auto listed ~$204 COMC; PSA 8 discount; Ray Allen HOF steady demand</t>
+          <t>Listed ~$204 COMC; PSA 8 discount</t>
         </is>
       </c>
     </row>
@@ -2756,10 +2756,10 @@
         <v>34</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>4.882352941176471</v>
+        <v>3.411764705882353</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
@@ -2768,12 +2768,12 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Yao low-numbered Panini inserts (Optic Gold /10 PSA 10) list $150-300; Crusade desirable insert</t>
+          <t>HOF; low-numbered insert</t>
         </is>
       </c>
     </row>
@@ -2795,10 +2795,10 @@
         <v>16</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>36.5</v>
+        <v>30.25</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2807,12 +2807,12 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>CSG 9.5 copies listed ~$970 retail; BGS 9.5 slight premium; sold likely $500-700</t>
+          <t>CSG 9.5 listed ~$970; BGS 9.5 comparable</t>
         </is>
       </c>
     </row>
@@ -2846,12 +2846,12 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Med-High</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>PSA auction: 2024 VIP Gold CC PSA 8 sold $75 on eBay (Jan 2025)</t>
+          <t>Sold $75 Jan 2025</t>
         </is>
       </c>
     </row>
@@ -2873,10 +2873,10 @@
         <v>26</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>5.730769230769231</v>
+        <v>4.769230769230769</v>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
@@ -2885,12 +2885,12 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Banchero autos /25-75 mid-tier products $100-250; PSA 8 card grade notable discount</t>
+          <t>Banchero numbered autos $100-250</t>
         </is>
       </c>
     </row>
@@ -2912,10 +2912,10 @@
         <v>52</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>1.403846153846154</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Panini Instant auto /99 draft night cards sold $100-150 raw on eBay; #3 pick</t>
+          <t>Instant auto /99 draft cards $100-150</t>
         </is>
       </c>
     </row>
@@ -2951,10 +2951,10 @@
         <v>75</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>4.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
@@ -2963,12 +2963,12 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Low-Med</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Penmanship Purple Ice /99 PSA 10 comps strong; Blue Ice /75 scarcer; SGC 10/10 premium</t>
+          <t>Prospect; Blue Ice scarcer than Purple</t>
         </is>
       </c>
     </row>
@@ -2990,10 +2990,10 @@
         <v>22</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
@@ -3002,12 +3002,12 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Raw Bowman U Purple /25 sold ~$11.50; PSA 9 ~3-4x raw; women's cards soft outside CC</t>
+          <t>Raw sold $11.50; PSA 9 bump modest</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -3042,7 +3042,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Total Cards Analyzed</t>
+          <t>Total Cards</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -3062,11 +3062,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total Est. FMV</t>
+          <t>Total Conservative FMV</t>
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>51860</v>
+        <v>55695</v>
       </c>
     </row>
     <row r="6">
@@ -3077,9 +3077,13 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>106.9%</t>
-        </is>
-      </c>
+          <t>122.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3098,7 +3102,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3108,7 +3112,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -3118,307 +3122,78 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
-      </c>
-    </row>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>TOP VALUE PLAYS (by upside %)</t>
-        </is>
-      </c>
+      <c r="A13" s="15" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Card</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>FMV</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>Upside</t>
-        </is>
-      </c>
+      <c r="A14" s="16" t="n"/>
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="16" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Mantle/Ruth/Gehrig Flawless Triple /15 PSA 10 Pop 2</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="n">
-        <v>1601</v>
-      </c>
-      <c r="C15" s="14" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>400%</t>
-        </is>
-      </c>
+      <c r="B15" s="14" t="n"/>
+      <c r="C15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Curry Kaleidoscopic Gold /10 PSA 10 Pop 4</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="n">
-        <v>1400</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>6000</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>329%</t>
-        </is>
-      </c>
+      <c r="B16" s="14" t="n"/>
+      <c r="C16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Curry VIP Gold Memorabilia /5 BGS 8</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="n">
-        <v>14</v>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>257%</t>
-        </is>
-      </c>
+      <c r="B17" s="14" t="n"/>
+      <c r="C17" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Curry NT Clutch Factor /25 PSA 9 Pop 4</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n">
-        <v>803</v>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>211%</t>
-        </is>
-      </c>
+      <c r="B18" s="14" t="n"/>
+      <c r="C18" s="14" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Ray Allen Immaculate Ink Red /25 PSA 8</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C19" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>200%</t>
-        </is>
-      </c>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>SGA Immaculate Gold Patch Auto /10</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="n">
-        <v>450</v>
-      </c>
-      <c r="C20" s="14" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>167%</t>
-        </is>
-      </c>
+      <c r="B20" s="14" t="n"/>
+      <c r="C20" s="14" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Shaq NT 1/1 Lasting Legacies Patch Auto</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="n">
-        <v>1588</v>
-      </c>
-      <c r="C21" s="14" t="n">
-        <v>4000</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>152%</t>
-        </is>
-      </c>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>SGA NT Viewpoint Emerald /5</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="n">
-        <v>600</v>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>150%</t>
-        </is>
-      </c>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Yao Pristine Refractor BGS 9.5</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="n">
-        <v>16</v>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>40</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>150%</t>
-        </is>
-      </c>
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Luka Prizm Mojo Auto /25</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="n">
-        <v>810</v>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>147%</t>
-        </is>
-      </c>
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Giannis Flawless Premium Ink /25 BGS 9.5/10</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="n">
-        <v>155</v>
-      </c>
-      <c r="C25" s="14" t="n">
-        <v>350</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>126%</t>
-        </is>
-      </c>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Luka Courtside Gold /10 PSA 9</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="n">
-        <v>362</v>
-      </c>
-      <c r="C26" s="14" t="n">
-        <v>800</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>121%</t>
-        </is>
-      </c>
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="14" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Curry One &amp; One /25 BGS 9/10 Pop 3</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="n">
-        <v>160</v>
-      </c>
-      <c r="C27" s="14" t="n">
-        <v>350</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>119%</t>
-        </is>
-      </c>
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Chet Flawless Excellence 1/1 Auto</t>
-        </is>
-      </c>
-      <c r="B28" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>250</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>108%</t>
-        </is>
-      </c>
+      <c r="B28" s="14" t="n"/>
+      <c r="C28" s="14" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Hannah Hidalgo Bowman U Purple /25 PSA 9</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n">
-        <v>22</v>
-      </c>
-      <c r="C29" s="14" t="n">
-        <v>45</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>105%</t>
-        </is>
-      </c>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update #15 SGA NT Viewpoint Emerald /5 - confirmed AUTO
FMV $475->$1,500. Moved from PASS to STRONG BUY. SGA /5 NT auto
of reigning MVP is premium card, not a base insert.

https://claude.ai/code/session_01GTThiDtMm869wgd52PwWVn
</commit_message>
<xml_diff>
--- a/Inventory/Goldin_Auction_FMV.xlsx
+++ b/Inventory/Goldin_Auction_FMV.xlsx
@@ -1157,14 +1157,14 @@
         <v>600</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>475</v>
-      </c>
-      <c r="F16" s="9" t="n">
-        <v>-0.2083333333333333</v>
-      </c>
-      <c r="G16" s="18" t="inlineStr">
-        <is>
-          <t>PASS</t>
+        <v>1500</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Listed $475; secondary insert not RPA</t>
+          <t>AUTO confirmed; SGA NT Emerald /5 auto; MVP candidate; NT premium over Immaculate</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -3081,10 +3081,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -3125,7 +3122,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="15" t="n"/>
     </row>

</xml_diff>

<commit_message>
Update #21 Jokic One & One Blue /49 - confirmed First Team AUTO
FMV $200->$800. Moved from PASS to STRONG BUY. Jokic 3x MVP auto
from One and One premium product. Max bid $625.

https://claude.ai/code/session_01GTThiDtMm869wgd52PwWVn
</commit_message>
<xml_diff>
--- a/Inventory/Goldin_Auction_FMV.xlsx
+++ b/Inventory/Goldin_Auction_FMV.xlsx
@@ -1391,14 +1391,14 @@
         <v>235</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>-0.148936170212766</v>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>800</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>2.404255319148936</v>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Non-auto; /49 base parallel</t>
+          <t>AUTO confirmed; First Team auto /49; Jokic 3x MVP; One and One premium product</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update #25 Giannis Select Tie-Dye /25 - confirmed AUTO
FMV $800->$1,500. BGS 9.5/10 auto in most popular Select parallel.
Max bid $1,200. Moved to snipe timing.

https://claude.ai/code/session_01GTThiDtMm869wgd52PwWVn
</commit_message>
<xml_diff>
--- a/Inventory/Goldin_Auction_FMV.xlsx
+++ b/Inventory/Goldin_Auction_FMV.xlsx
@@ -1547,10 +1547,10 @@
         <v>340</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>1.352941176470588</v>
+        <v>3.411764705882353</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Need to know if auto; if not, much less</t>
+          <t>AUTO confirmed; Select Tie-Dye /25 auto BGS 9.5/10; Giannis; most popular Select parallel</t>
         </is>
       </c>
     </row>

</xml_diff>